<commit_message>
Uploaded updated test files
</commit_message>
<xml_diff>
--- a/Tests/tests.xlsx
+++ b/Tests/tests.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\salma\Teaching\Concepts\Projects2026\Prolog_Starter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\salma.el-sayed\Concepts\Project_Prolog_Starter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231D9C64-DCE1-497D-BB03-2E067C02EB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{D783000B-55DF-493E-99E6-34911BD7F86F}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="25815" windowHeight="15495"/>
   </bookViews>
   <sheets>
-    <sheet name="public" sheetId="1" r:id="rId1"/>
+    <sheet name="public_fixed" sheetId="3" r:id="rId1"/>
     <sheet name="sample" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
   <si>
     <t>predicate</t>
   </si>
@@ -57,45 +56,16 @@
     <t>group_ingredients</t>
   </si>
   <si>
-    <t>schedule_all_reservations([day(1, 3), day(2, 3), day(5, 3)], [res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, evening_rush1, medium), res(day(1, 3), evening, evening_rush2, xlarge), res(day(2, 3), evening, f, xlarge), res(day(1, 3), morning, morning_rush1, large), res(day(2, 3), morning, morning_rush2, medium)]).</t>
-  </si>
-  <si>
     <t>schedule_all_reservations([day(1, 3)], R).</t>
   </si>
   <si>
     <t>the groups cannot all be fit into a single day</t>
   </si>
   <si>
-    <t>schedule_all_reservations([day(1, 3), day(2, 3), day(5, 3)],[res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, evening_rush1, medium), res(day(1, 3), evening, evening_rush2, xlarge), res(day(2, 3), evening, f, medium), res(day(1, 3), morning, morning_rush1, large), res(day(2, 3), morning, morning_rush2, medium)]).</t>
-  </si>
-  <si>
     <t>group f is assigned to medium table</t>
   </si>
   <si>
-    <t>schedule_all_reservations([day(1, 3), day(2, 3), day(5, 3)], R).</t>
-  </si>
-  <si>
-    <t>R = [res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, evening_rush1, medium), res(day(1, 3), evening, evening_rush2, xlarge), res(day(2, 3), evening, f, xlarge), res(day(1, 3), morning, morning_rush1, large), res(day(2, 3), morning, morning_rush2, medium)] ;
-R = [res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, evening_rush1, medium), res(day(1, 3), evening, evening_rush2, xlarge), res(day(2, 3), evening, f, xlarge), res(day(1, 3), morning, morning_rush1, large), res(day(2, 3), morning, morning_rush2, large)] ;
-R = [res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, evening_rush1, medium), res(day(1, 3), evening, evening_rush2, xlarge), res(day(2, 3), evening, f, xlarge), res(day(1, 3), morning, morning_rush1, large), res(day(2, 3), morning, morning_rush2, xlarge)]</t>
-  </si>
-  <si>
     <t>schedule_all_reservations([day(2, 3), day(4, 3)], R).</t>
-  </si>
-  <si>
-    <t>R = [res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, evening_rush1, medium), res(day(4, 3), evening, evening_rush2, large), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, morning_rush1, medium), res(day(4, 3), morning, morning_rush2, large)] ;
-R = [res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, evening_rush1, medium), res(day(4, 3), evening, evening_rush2, large), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, morning_rush1, large), res(day(4, 3), morning, morning_rush2, medium)] ;
-R = [res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, evening_rush1, large), res(day(4, 3), evening, evening_rush2, medium), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, morning_rush1, medium), res(day(4, 3), morning, morning_rush2, large)] ;
-R = [res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, evening_rush1, large), res(day(4, 3), evening, evening_rush2, medium), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, morning_rush1, large), res(day(4, 3), morning, morning_rush2, medium)]</t>
-  </si>
-  <si>
-    <t>check_staff(day(3, 3), morning,[res(day(3, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(3, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(3, 3), morning, e, xlarge), res(day(1, 3), evening, evening_rush1, medium), res(day(1, 3), evening, evening_rush2, xlarge), res(day(2, 3), evening, f, medium), res(day(1, 3), morning, morning_rush1, large), res(day(2, 3), morning, morning_rush2, medium)]).</t>
-  </si>
-  <si>
-    <t>check_staff(day(1, 3), morning,[res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, evening_rush1, medium), res(day(1, 3), evening, evening_rush2, xlarge), res(day(2, 3), evening, f, medium), res(day(1, 3), morning, morning_rush1, large), res(day(2, 3), morning, morning_rush2, medium)]).</t>
-  </si>
-  <si>
-    <t>check_staff(day(4, 3), morning,[res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, evening_rush1, medium), res(day(1, 3), evening, evening_rush2, xlarge), res(day(2, 3), evening, f, medium), res(day(1, 3), morning, morning_rush1, large), res(day(2, 3), morning, morning_rush2, medium)]).</t>
   </si>
   <si>
     <t xml:space="preserve"> needed_ingredients([res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, g, medium), res(day(4, 3), morning, h, large), res(day(4, 3), evening, i, medium), res(day(4, 3), evening, j, large)],   [(day(2, 3), [basil, cheese, chocolate, cucumber, eggs, flour, lettuce, olive_oil, salt, sugar, tomato]),  (day(4, 3), [basil, beef, broth, bun, butter, cheese, chocolate, cucumber, eggs, flour, garlic, herbs, lemon, lettuce, olive_oil, salmon, salt, sugar, tomato, vegetables])]).</t>
@@ -200,12 +170,33 @@
   <si>
     <t>I = [ing5, ing6, ing5, ing6, ing5, ing6, ing5, ing6]</t>
   </si>
+  <si>
+    <t>schedule_all_reservations([day(1, 3), day(2, 3), day(5, 3)], [res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, i, medium), res(day(1, 3), evening, j, xlarge), res(day(2, 3), evening, f, xlarge), res(day(1, 3), morning, g, large), res(day(2, 3), morning, h, medium)]).</t>
+  </si>
+  <si>
+    <t>schedule_all_reservations([day(1, 3), day(2, 3), day(5, 3)],[res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, i, medium), res(day(1, 3), evening, j, xlarge), res(day(2, 3), evening, f, medium), res(day(1, 3), morning, g, large), res(day(2, 3), morning, h, medium)]).</t>
+  </si>
+  <si>
+    <t>R = [res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, i, medium), res(day(4, 3), evening, j, large), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, g, medium), res(day(4, 3), morning, h, large)] ;
+R = [res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, i, medium), res(day(4, 3), evening, j, large), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, g, large), res(day(4, 3), morning, h, medium)] ;
+R = [res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, i, large), res(day(4, 3), evening, j, medium), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, g, medium), res(day(4, 3), morning, h, large)] ;
+R = [res(day(2, 3), morning, a, small), res(day(2, 3), evening, b, small), res(day(2, 3), morning, c, medium), res(day(2, 3), evening, d, large), res(day(4, 3), morning, e, xlarge), res(day(4, 3), evening, i, large), res(day(4, 3), evening, j, medium), res(day(4, 3), evening, f, xlarge), res(day(4, 3), morning, g, large), res(day(4, 3), morning, h, medium)]</t>
+  </si>
+  <si>
+    <t>check_staff(day(3, 3), morning,[res(day(3, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(3, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(3, 3), morning, e, xlarge), res(day(1, 3), evening, i, medium), res(day(1, 3), evening, j, xlarge), res(day(2, 3), evening, f, medium), res(day(1, 3), morning, g, large), res(day(2, 3), morning, h, medium)]).</t>
+  </si>
+  <si>
+    <t>check_staff(day(1, 3), morning,[res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, i, medium), res(day(1, 3), evening, j, xlarge), res(day(2, 3), evening, f, medium), res(day(1, 3), morning, g, large), res(day(2, 3), morning, h, medium)]).</t>
+  </si>
+  <si>
+    <t>check_staff(day(4, 3), morning,[res(day(1, 3), morning, a, small), res(day(1, 3), evening, b, small), res(day(1, 3), morning, c, medium), res(day(1, 3), evening, d, large), res(day(1, 3), morning, e, xlarge), res(day(1, 3), evening, i, medium), res(day(1, 3), evening, j, xlarge), res(day(2, 3), evening, f, medium), res(day(1, 3), morning, g, large), res(day(2, 3), morning, h, medium)]).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,6 +308,33 @@
   </cellStyles>
   <dxfs count="7">
     <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFAB0B0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
@@ -356,33 +374,6 @@
         <horizontal/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFAB0B0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -397,26 +388,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0EBBA2D0-E301-4F61-8B0C-A9E8C994D701}" name="Table1" displayName="Table1" ref="A1:D1048576" totalsRowShown="0">
-  <autoFilter ref="A1:D1048576" xr:uid="{0EBBA2D0-E301-4F61-8B0C-A9E8C994D701}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table15" displayName="Table15" ref="A1:D1048575" totalsRowShown="0">
+  <autoFilter ref="A1:D1048575"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{CFF98AE4-4A31-4723-87D0-A48F95D5DD27}" name="predicate"/>
-    <tableColumn id="2" xr3:uid="{EBD00AD5-2259-444A-B136-D7B3C87D8F51}" name="query"/>
-    <tableColumn id="3" xr3:uid="{9F34B1CF-CEE7-4E7B-9529-B1C8171FF2A0}" name="ouput/sample outputs" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{744BC17C-9AE8-4926-83EC-D5DEB6E68B3C}" name="explanation"/>
+    <tableColumn id="1" name="predicate"/>
+    <tableColumn id="2" name="query"/>
+    <tableColumn id="3" name="ouput/sample outputs" dataDxfId="3"/>
+    <tableColumn id="4" name="explanation"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C45E5A9A-B71A-466F-A6EC-C9EDA2A2F16E}" name="Table2" displayName="Table2" ref="A1:D10" totalsRowShown="0">
-  <autoFilter ref="A1:D10" xr:uid="{C45E5A9A-B71A-466F-A6EC-C9EDA2A2F16E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:D10" totalsRowShown="0">
+  <autoFilter ref="A1:D10"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2C67B828-0B2B-4FBB-951C-BA214AF7DE15}" name="predicate" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{84134F1C-7A43-4657-8170-0F5C6F4DCF61}" name="query" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{D91D683D-0DC7-464C-A765-7B47A4C77D5E}" name="ouput/sample outputs" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{53F02070-6339-4BCD-9A63-0B8F37EDE8F1}" name="explanation"/>
+    <tableColumn id="1" name="predicate" dataDxfId="6"/>
+    <tableColumn id="2" name="query" dataDxfId="5"/>
+    <tableColumn id="3" name="ouput/sample outputs" dataDxfId="4"/>
+    <tableColumn id="4" name="explanation"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -738,17 +729,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EC23FF2-7D49-419D-A7C0-480F709D00C3}">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="80.81640625" customWidth="1"/>
-    <col min="3" max="3" width="69.6328125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="80.875" customWidth="1"/>
+    <col min="3" max="3" width="69.625" style="7" customWidth="1"/>
     <col min="4" max="4" width="53" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -756,205 +747,193 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="71.25">
       <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="C2" s="6" t="b">
         <v>1</v>
       </c>
       <c r="D2" s="5"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="6" t="b">
         <v>0</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="71.25">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="C4" s="6" t="b">
         <v>0</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="217.5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="285">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" spans="1:4" ht="290" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" ht="71.25">
       <c r="A6" s="5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>14</v>
+        <v>45</v>
+      </c>
+      <c r="C6" s="6" t="b">
+        <v>0</v>
       </c>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="71.25">
       <c r="A7" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="C7" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="71.25">
       <c r="A8" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="C8" s="6" t="b">
         <v>1</v>
       </c>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="99.75">
       <c r="A9" s="5" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C9" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="5"/>
-    </row>
-    <row r="10" spans="1:4" ht="101.5" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="185.25">
       <c r="A10" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="188.5" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="1:4" ht="213.75">
       <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>21</v>
+        <v>14</v>
+      </c>
+      <c r="C11" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" spans="1:4" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="28.5">
       <c r="A12" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="6" t="b">
-        <v>1</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="C12" s="6"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="28.5">
       <c r="A13" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="6"/>
+        <v>16</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>17</v>
+      </c>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4">
       <c r="A14" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="D14" s="5"/>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D15" s="5"/>
+    </row>
+    <row r="16" spans="1:4" ht="28.5">
+      <c r="A16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="5"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="5"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>32</v>
-      </c>
       <c r="D16" s="5"/>
-    </row>
-    <row r="17" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -965,17 +944,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0281CE3E-4629-417B-973A-A73BFCADB379}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="62.6328125" customWidth="1"/>
-    <col min="3" max="3" width="66.26953125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="51.90625" customWidth="1"/>
+    <col min="2" max="2" width="62.625" customWidth="1"/>
+    <col min="3" max="3" width="66.25" style="7" customWidth="1"/>
+    <col min="4" max="4" width="51.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -983,129 +962,129 @@
         <v>1</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="42.75">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C2" s="2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C3" s="2" t="b">
         <v>0</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="232" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="228">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="28.5">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="28.5">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="42.75">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="71.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2" t="b">
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C9" s="2" t="b">
         <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:C6 B5">
-    <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",B5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",B5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1122,7 +1101,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:B10 B7">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="sample">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="sample">
       <formula>NOT(ISERROR(SEARCH("sample",B7)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>